<commit_message>
#7 Changes Completed and deliverables Generated.
</commit_message>
<xml_diff>
--- a/Design-Files/Main-Controller-Board-v1.2.0/BOM/Client-BOM_Main-Controller-Board-v1.2.0.xlsx
+++ b/Design-Files/Main-Controller-Board-v1.2.0/BOM/Client-BOM_Main-Controller-Board-v1.2.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="178">
   <si>
     <t>#</t>
   </si>
@@ -45,9 +45,6 @@
     <t>Connector</t>
   </si>
   <si>
-    <t>Headers and Wire Housings</t>
-  </si>
-  <si>
     <t>Inductor</t>
   </si>
   <si>
@@ -129,9 +126,6 @@
     <t>J3</t>
   </si>
   <si>
-    <t>J5</t>
-  </si>
-  <si>
     <t>L1</t>
   </si>
   <si>
@@ -231,9 +225,6 @@
     <t>1x6P SH 1 1mm 6 SMD,P=1mm Wire To Board / Wire To Wire Connector ROHS</t>
   </si>
   <si>
-    <t>1x4P 4P XH Tin 4 -25℃~+85℃ 3A 1 2.5mm Brass Bend insert Push-Pull,P=2.5mm Wire To Board Connector ROHS</t>
-  </si>
-  <si>
     <t>2.26A 4.7uH ±20% SMD,7.3x7.3mm Power Inductors ROHS</t>
   </si>
   <si>
@@ -318,9 +309,6 @@
     <t>DC-044K-D025</t>
   </si>
   <si>
-    <t>S4B-XH-A(LF)(SN)</t>
-  </si>
-  <si>
     <t>YPRH0703-4R7M</t>
   </si>
   <si>
@@ -469,9 +457,6 @@
   </si>
   <si>
     <t>BOOMELE</t>
-  </si>
-  <si>
-    <t>JST</t>
   </si>
   <si>
     <t>YJYCOIN</t>
@@ -786,9 +771,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -797,6 +779,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1085,7 +1070,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -1109,9 +1094,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1122,28 +1107,28 @@
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1154,22 +1139,22 @@
       </c>
       <c r="C3" s="12"/>
       <c r="D3" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="J3" s="7">
         <v>2</v>
@@ -1179,29 +1164,29 @@
     <row r="4" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B36" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B35" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="13" t="s">
         <v>2</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="J4" s="9">
         <v>2</v>
@@ -1218,22 +1203,22 @@
         <v>2</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="J5" s="7">
         <v>3</v>
@@ -1250,22 +1235,22 @@
         <v>3</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="J6" s="9">
         <v>1</v>
@@ -1280,22 +1265,22 @@
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="J7" s="7">
         <v>1</v>
@@ -1312,22 +1297,22 @@
         <v>2</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="J8" s="9">
         <v>1</v>
@@ -1342,22 +1327,22 @@
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
@@ -1374,22 +1359,22 @@
         <v>2</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="J10" s="9">
         <v>3</v>
@@ -1406,22 +1391,22 @@
         <v>3</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="J11" s="7">
         <v>3</v>
@@ -1438,22 +1423,22 @@
         <v>3</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
@@ -1470,22 +1455,22 @@
         <v>4</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
@@ -1502,22 +1487,22 @@
         <v>4</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="J14" s="9">
         <v>1</v>
@@ -1534,22 +1519,22 @@
         <v>5</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -1566,22 +1551,22 @@
         <v>6</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="J16" s="9">
         <v>1</v>
@@ -1597,29 +1582,29 @@
       <c r="C17" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D17" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="E17" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="F17" s="15" t="s">
-        <v>181</v>
-      </c>
-      <c r="G17" s="16" t="s">
-        <v>123</v>
-      </c>
-      <c r="H17" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="I17" s="16" t="s">
-        <v>168</v>
-      </c>
-      <c r="J17" s="15">
+      <c r="D17" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="E17" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="G17" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="H17" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="I17" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="J17" s="14">
         <v>1</v>
       </c>
-      <c r="K17" s="17" t="s">
-        <v>182</v>
+      <c r="K17" s="16" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1632,601 +1617,569 @@
         <v>7</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
       </c>
       <c r="K18" s="9"/>
     </row>
-    <row r="19" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
-        <f>ROW(B19) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="C19" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="D19" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>70</v>
+      <c r="D19" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>68</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>181</v>
-      </c>
-      <c r="G19" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="I19" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="J19" s="7">
+        <v>176</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="I19" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="J19" s="9">
         <v>1</v>
       </c>
-      <c r="K19" s="7"/>
+      <c r="K19" s="9"/>
     </row>
     <row r="20" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B20) - ROW($B$2)</f>
         <v>18</v>
       </c>
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D20" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>71</v>
+      <c r="D20" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>69</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>181</v>
-      </c>
-      <c r="G20" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="H20" s="9" t="s">
-        <v>151</v>
-      </c>
-      <c r="I20" s="10" t="s">
-        <v>169</v>
-      </c>
-      <c r="J20" s="9">
+        <v>97</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="I20" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="J20" s="7">
         <v>1</v>
       </c>
-      <c r="K20" s="9"/>
-    </row>
-    <row r="21" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K20" s="7"/>
+    </row>
+    <row r="21" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="11">
-        <f>ROW(B21) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C21" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="D21" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="E21" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="G21" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="H21" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="I21" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="J21" s="7">
-        <v>1</v>
-      </c>
-      <c r="K21" s="7"/>
-    </row>
-    <row r="22" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D21" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="G21" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="I21" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="J21" s="9">
+        <v>6</v>
+      </c>
+      <c r="K21" s="9"/>
+    </row>
+    <row r="22" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B22) - ROW($B$2)</f>
         <v>20</v>
       </c>
-      <c r="C22" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="G22" s="10" t="s">
-        <v>125</v>
-      </c>
-      <c r="H22" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="I22" s="10" t="s">
-        <v>180</v>
-      </c>
-      <c r="J22" s="9">
-        <v>6</v>
-      </c>
-      <c r="K22" s="9"/>
-    </row>
-    <row r="23" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C22" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="I22" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="J22" s="7">
+        <v>3</v>
+      </c>
+      <c r="K22" s="7"/>
+    </row>
+    <row r="23" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
-        <f>ROW(B23) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="C23" s="12" t="s">
+      <c r="C23" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D23" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E23" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="G23" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="H23" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="I23" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="J23" s="7">
+      <c r="D23" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E23" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="G23" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="I23" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="J23" s="9">
         <v>3</v>
       </c>
-      <c r="K23" s="7"/>
+      <c r="K23" s="9"/>
     </row>
     <row r="24" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B24) - ROW($B$2)</f>
         <v>22</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C24" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="D24" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="E24" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="G24" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="H24" s="9" t="s">
-        <v>155</v>
-      </c>
-      <c r="I24" s="10" t="s">
-        <v>180</v>
-      </c>
-      <c r="J24" s="9">
-        <v>3</v>
-      </c>
-      <c r="K24" s="9"/>
+      <c r="D24" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="I24" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="J24" s="7">
+        <v>2</v>
+      </c>
+      <c r="K24" s="7"/>
     </row>
     <row r="25" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="11">
-        <f>ROW(B25) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="C25" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="G25" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="H25" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="I25" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="J25" s="7">
-        <v>2</v>
-      </c>
-      <c r="K25" s="7"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="G25" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="H25" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="I25" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="J25" s="9">
+        <v>4</v>
+      </c>
+      <c r="K25" s="9"/>
     </row>
     <row r="26" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B26) - ROW($B$2)</f>
         <v>24</v>
       </c>
-      <c r="C26" s="13"/>
-      <c r="D26" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E26" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="F26" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="G26" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="H26" s="9" t="s">
-        <v>142</v>
-      </c>
-      <c r="I26" s="10" t="s">
-        <v>171</v>
-      </c>
-      <c r="J26" s="9">
-        <v>4</v>
-      </c>
-      <c r="K26" s="9"/>
+      <c r="C26" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="G26" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="I26" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="J26" s="7">
+        <v>1</v>
+      </c>
+      <c r="K26" s="7"/>
     </row>
     <row r="27" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="11">
-        <f>ROW(B27) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="C27" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="D27" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="E27" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="G27" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="H27" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="I27" s="8" t="s">
-        <v>172</v>
-      </c>
-      <c r="J27" s="7">
+      <c r="C27" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="G27" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="H27" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="I27" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="J27" s="9">
         <v>1</v>
       </c>
-      <c r="K27" s="7"/>
+      <c r="K27" s="9"/>
     </row>
     <row r="28" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B28) - ROW($B$2)</f>
         <v>26</v>
       </c>
-      <c r="C28" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="E28" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F28" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="G28" s="10" t="s">
-        <v>131</v>
-      </c>
-      <c r="H28" s="9" t="s">
-        <v>142</v>
-      </c>
-      <c r="I28" s="10" t="s">
-        <v>173</v>
-      </c>
-      <c r="J28" s="9">
-        <v>1</v>
-      </c>
-      <c r="K28" s="9"/>
-    </row>
-    <row r="29" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C28" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="G28" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="I28" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="J28" s="7">
+        <v>6</v>
+      </c>
+      <c r="K28" s="7"/>
+    </row>
+    <row r="29" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
-        <f>ROW(B29) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="C29" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="E29" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="G29" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="H29" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="I29" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="J29" s="7">
-        <v>6</v>
-      </c>
-      <c r="K29" s="7"/>
-    </row>
-    <row r="30" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C29" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="G29" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="H29" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="I29" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="J29" s="9">
+        <v>3</v>
+      </c>
+      <c r="K29" s="9"/>
+    </row>
+    <row r="30" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B30) - ROW($B$2)</f>
         <v>28</v>
       </c>
-      <c r="C30" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D30" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="E30" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="F30" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="G30" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="H30" s="9" t="s">
-        <v>156</v>
-      </c>
-      <c r="I30" s="10" t="s">
-        <v>175</v>
-      </c>
-      <c r="J30" s="9">
+      <c r="C30" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="I30" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="J30" s="7">
         <v>3</v>
       </c>
-      <c r="K30" s="9"/>
+      <c r="K30" s="7"/>
     </row>
     <row r="31" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="11">
-        <f>ROW(B31) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C31" s="12" t="s">
+      <c r="C31" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D31" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="E31" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="G31" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="H31" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="I31" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="J31" s="7">
-        <v>3</v>
-      </c>
-      <c r="K31" s="7"/>
+      <c r="D31" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E31" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="G31" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="I31" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="J31" s="9">
+        <v>2</v>
+      </c>
+      <c r="K31" s="9"/>
     </row>
     <row r="32" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B32) - ROW($B$2)</f>
         <v>30</v>
       </c>
-      <c r="C32" s="13" t="s">
+      <c r="C32" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="D32" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="E32" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="F32" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="G32" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="H32" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="I32" s="10" t="s">
-        <v>180</v>
-      </c>
-      <c r="J32" s="9">
-        <v>2</v>
-      </c>
-      <c r="K32" s="9"/>
-    </row>
-    <row r="33" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D32" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="G32" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="I32" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="J32" s="7">
+        <v>1</v>
+      </c>
+      <c r="K32" s="7"/>
+    </row>
+    <row r="33" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="11">
-        <f>ROW(B33) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="C33" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="D33" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="E33" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="F33" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="G33" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="H33" s="7" t="s">
+      <c r="C33" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E33" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="G33" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="H33" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="I33" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="J33" s="7">
+      <c r="I33" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="J33" s="9">
         <v>1</v>
       </c>
-      <c r="K33" s="7"/>
-    </row>
-    <row r="34" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K33" s="9"/>
+    </row>
+    <row r="34" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="11">
-        <f t="shared" si="0"/>
+        <f>ROW(B34) - ROW($B$2)</f>
         <v>32</v>
       </c>
-      <c r="C34" s="13" t="s">
+      <c r="C34" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="D34" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E34" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="F34" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="G34" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="H34" s="9" t="s">
-        <v>158</v>
-      </c>
-      <c r="I34" s="10" t="s">
-        <v>180</v>
-      </c>
-      <c r="J34" s="9">
+      <c r="D34" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="G34" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="H34" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="I34" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="J34" s="7">
         <v>1</v>
       </c>
-      <c r="K34" s="9"/>
-    </row>
-    <row r="35" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K34" s="7"/>
+    </row>
+    <row r="35" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="11">
-        <f>ROW(B35) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="C35" s="12" t="s">
+      <c r="C35" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="D35" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="F35" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="G35" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="H35" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="I35" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="J35" s="7">
-        <v>1</v>
-      </c>
-      <c r="K35" s="7"/>
-    </row>
-    <row r="36" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="1"/>
-      <c r="B36" s="11">
-        <f t="shared" si="0"/>
-        <v>34</v>
-      </c>
-      <c r="C36" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D36" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="E36" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="G36" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="H36" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="I36" s="10" t="s">
-        <v>180</v>
-      </c>
-      <c r="J36" s="9">
+      <c r="D35" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="E35" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="G35" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="H35" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="I35" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="J35" s="9">
         <v>3</v>
       </c>
-      <c r="K36" s="9"/>
+      <c r="K35" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>